<commit_message>
Update to KiCAD 9 Fixed Ultrasonic sensor footprint
</commit_message>
<xml_diff>
--- a/Seznam_komponent.xlsx
+++ b/Seznam_komponent.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t xml:space="preserve">U Martina</t>
   </si>
@@ -39,10 +39,7 @@
     <t xml:space="preserve">H-bridge DRV8833</t>
   </si>
   <si>
-    <t xml:space="preserve">Sada 2ks kol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sada 2ks motorků</t>
+    <t xml:space="preserve">Sada 2ks kol a motorů</t>
   </si>
   <si>
     <t xml:space="preserve">Vypínač</t>
@@ -54,7 +51,7 @@
     <t xml:space="preserve">USB konektory</t>
   </si>
   <si>
-    <t xml:space="preserve">IR čidla sada 5ks</t>
+    <t xml:space="preserve">IR čidlo 8ch</t>
   </si>
   <si>
     <t xml:space="preserve">USB mikro kabel</t>
@@ -102,16 +99,28 @@
     <t xml:space="preserve">M3x14</t>
   </si>
   <si>
+    <t xml:space="preserve">Napětí</t>
+  </si>
+  <si>
     <t xml:space="preserve">M3x20</t>
   </si>
   <si>
+    <t xml:space="preserve">Proud</t>
+  </si>
+  <si>
     <t xml:space="preserve">M3x25</t>
   </si>
   <si>
+    <t xml:space="preserve">Odpor</t>
+  </si>
+  <si>
     <t xml:space="preserve">M3x30</t>
   </si>
   <si>
     <t xml:space="preserve">4  ks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Výkon</t>
   </si>
   <si>
     <t xml:space="preserve">M3n</t>
@@ -218,10 +227,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F36"/>
-  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:I36"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.86"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -229,7 +240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="0" t="s">
         <v>1</v>
       </c>
@@ -254,7 +265,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
         <v>3</v>
       </c>
@@ -279,7 +290,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
         <v>5</v>
       </c>
@@ -290,192 +301,188 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>9</v>
+        <v>15</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="0" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D8" s="0" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="0" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" s="0" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F9" s="0" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>20</v>
+        <v>13</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="F10" s="0" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>13</v>
-      </c>
-      <c r="D11" s="0" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F11" s="0" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="0" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="0" t="n">
-        <v>6</v>
-      </c>
       <c r="F13" s="0" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
         <v>14</v>
       </c>
       <c r="F15" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="0" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
         <v>16</v>
       </c>
+      <c r="C17" s="0" t="n">
+        <v>3</v>
+      </c>
       <c r="F17" s="0" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="0" t="n">
-        <v>3</v>
-      </c>
       <c r="F18" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
         <v>18</v>
       </c>
       <c r="F19" s="0" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
         <v>19</v>
       </c>
       <c r="F20" s="0" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="0" t="n">
         <v>50</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F24" s="0" t="n">
-        <f aca="false">SUM(F2:F23)</f>
-        <v>595</v>
-      </c>
-    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F23" s="0" t="n">
+        <f aca="false">SUM(F2:F22)</f>
+        <v>552</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="0" t="s">
         <v>21</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>23</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="H32" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>24</v>
+      <c r="I32" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -483,31 +490,50 @@
         <v>26</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="H33" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="0" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="H34" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="I34" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>29</v>
+        <v>31</v>
+      </c>
+      <c r="H35" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <f aca="false">I34*I33*I33</f>
+        <v>0.16</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +553,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -545,7 +571,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>